<commit_message>
:kiwi_fruit" alpha div. with new datasets + clearer labels for dataset 1 fig.
</commit_message>
<xml_diff>
--- a/data/derived_data/4_Diversities/ps_ITS_rare_expe_D1_tax_table.xlsx
+++ b/data/derived_data/4_Diversities/ps_ITS_rare_expe_D1_tax_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="249">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -119,9 +119,6 @@
     <t xml:space="preserve">Unknown</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_105</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_111</t>
   </si>
   <si>
@@ -134,7 +131,7 @@
     <t xml:space="preserve">Cluster_113</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_113</t>
+    <t xml:space="preserve">pulcherrima</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_116</t>
@@ -362,7 +359,22 @@
     <t xml:space="preserve">Cluster_240</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_240</t>
+    <t xml:space="preserve">Viridiplantae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Streptophyta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magnoliopsida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rosales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rosaceae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rubus</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_242</t>
@@ -467,9 +479,6 @@
     <t xml:space="preserve">Cluster_317</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_317</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_32</t>
   </si>
   <si>
@@ -485,9 +494,6 @@
     <t xml:space="preserve">Cluster_340</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_340</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_341</t>
   </si>
   <si>
@@ -527,7 +533,10 @@
     <t xml:space="preserve">Cluster_371</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_371</t>
+    <t xml:space="preserve">Prunus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avium</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_379</t>
@@ -587,9 +596,6 @@
     <t xml:space="preserve">Cluster_423</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_423</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_44</t>
   </si>
   <si>
@@ -650,15 +656,12 @@
     <t xml:space="preserve">Cluster_576</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_576</t>
+    <t xml:space="preserve">sulcatus</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_58</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_58</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_59</t>
   </si>
   <si>
@@ -677,9 +680,6 @@
     <t xml:space="preserve">Cluster_63</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_63</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_64</t>
   </si>
   <si>
@@ -698,18 +698,12 @@
     <t xml:space="preserve">Cluster_68</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_68</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_7</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_72</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_72</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_73</t>
   </si>
   <si>
@@ -734,15 +728,9 @@
     <t xml:space="preserve">Cluster_83</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_83</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_87</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_87</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_88</t>
   </si>
   <si>
@@ -752,9 +740,6 @@
     <t xml:space="preserve">Cluster_89</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown_89</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_9</t>
   </si>
   <si>
@@ -768,9 +753,6 @@
   </si>
   <si>
     <t xml:space="preserve">Cluster_95</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unknown_95</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_96</t>
@@ -1240,22 +1222,22 @@
         <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="H6" t="s">
         <v>34</v>
@@ -1263,7 +1245,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -1289,85 +1271,85 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" t="s">
         <v>37</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" t="s">
+        <v>19</v>
+      </c>
+      <c r="H9" t="s">
         <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" t="s">
-        <v>40</v>
-      </c>
-      <c r="H9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" t="s">
         <v>41</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
@@ -1388,12 +1370,12 @@
         <v>19</v>
       </c>
       <c r="H11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
         <v>9</v>
@@ -1414,30 +1396,30 @@
         <v>14</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
         <v>46</v>
       </c>
-      <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>47</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>48</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>49</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>50</v>
-      </c>
-      <c r="G13" t="s">
-        <v>51</v>
       </c>
       <c r="H13" t="s">
         <v>34</v>
@@ -1445,7 +1427,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
@@ -1471,7 +1453,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -1492,38 +1474,38 @@
         <v>19</v>
       </c>
       <c r="H15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
         <v>54</v>
       </c>
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>55</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>56</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>57</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>58</v>
-      </c>
-      <c r="H16" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
@@ -1535,13 +1517,13 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" t="s">
         <v>61</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>62</v>
-      </c>
-      <c r="G17" t="s">
-        <v>63</v>
       </c>
       <c r="H17" t="s">
         <v>34</v>
@@ -1549,7 +1531,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
         <v>9</v>
@@ -1570,12 +1552,12 @@
         <v>19</v>
       </c>
       <c r="H18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
         <v>9</v>
@@ -1596,30 +1578,30 @@
         <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" t="s">
         <v>66</v>
       </c>
-      <c r="B20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" t="s">
-        <v>48</v>
-      </c>
-      <c r="E20" t="s">
-        <v>49</v>
-      </c>
-      <c r="F20" t="s">
-        <v>67</v>
-      </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H20" t="s">
         <v>34</v>
@@ -1627,7 +1609,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
@@ -1639,21 +1621,21 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
+        <v>68</v>
+      </c>
+      <c r="F21" t="s">
         <v>69</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>70</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>71</v>
-      </c>
-      <c r="H21" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
@@ -1665,39 +1647,39 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
+        <v>60</v>
+      </c>
+      <c r="F22" t="s">
         <v>61</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>62</v>
       </c>
-      <c r="G22" t="s">
-        <v>63</v>
-      </c>
       <c r="H22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" t="s">
+        <v>34</v>
+      </c>
+      <c r="E23" t="s">
+        <v>34</v>
+      </c>
+      <c r="F23" t="s">
         <v>75</v>
       </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" t="s">
-        <v>34</v>
-      </c>
-      <c r="D23" t="s">
-        <v>34</v>
-      </c>
-      <c r="E23" t="s">
-        <v>34</v>
-      </c>
-      <c r="F23" t="s">
-        <v>76</v>
-      </c>
       <c r="G23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H23" t="s">
         <v>34</v>
@@ -1705,7 +1687,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
         <v>9</v>
@@ -1717,13 +1699,13 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F24" t="s">
         <v>61</v>
       </c>
-      <c r="F24" t="s">
-        <v>62</v>
-      </c>
       <c r="G24" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H24" t="s">
         <v>34</v>
@@ -1731,7 +1713,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
@@ -1757,7 +1739,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" t="s">
         <v>9</v>
@@ -1769,39 +1751,39 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" t="s">
         <v>61</v>
       </c>
-      <c r="F26" t="s">
-        <v>62</v>
-      </c>
       <c r="G26" t="s">
+        <v>80</v>
+      </c>
+      <c r="H26" t="s">
         <v>81</v>
-      </c>
-      <c r="H26" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" t="s">
+        <v>47</v>
+      </c>
+      <c r="E27" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" t="s">
         <v>83</v>
       </c>
-      <c r="B27" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" t="s">
-        <v>47</v>
-      </c>
-      <c r="D27" t="s">
-        <v>48</v>
-      </c>
-      <c r="E27" t="s">
-        <v>49</v>
-      </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>84</v>
-      </c>
-      <c r="G27" t="s">
-        <v>85</v>
       </c>
       <c r="H27" t="s">
         <v>34</v>
@@ -1809,25 +1791,25 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
+        <v>85</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" t="s">
+        <v>47</v>
+      </c>
+      <c r="E28" t="s">
+        <v>48</v>
+      </c>
+      <c r="F28" t="s">
         <v>86</v>
       </c>
-      <c r="B28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" t="s">
-        <v>47</v>
-      </c>
-      <c r="D28" t="s">
-        <v>48</v>
-      </c>
-      <c r="E28" t="s">
-        <v>49</v>
-      </c>
-      <c r="F28" t="s">
-        <v>87</v>
-      </c>
       <c r="G28" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H28" t="s">
         <v>34</v>
@@ -1835,7 +1817,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
@@ -1850,10 +1832,10 @@
         <v>29</v>
       </c>
       <c r="F29" t="s">
+        <v>88</v>
+      </c>
+      <c r="G29" t="s">
         <v>89</v>
-      </c>
-      <c r="G29" t="s">
-        <v>90</v>
       </c>
       <c r="H29" t="s">
         <v>34</v>
@@ -1861,25 +1843,25 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
+        <v>90</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>34</v>
+      </c>
+      <c r="D30" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30" t="s">
+        <v>34</v>
+      </c>
+      <c r="F30" t="s">
         <v>91</v>
       </c>
-      <c r="B30" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" t="s">
-        <v>34</v>
-      </c>
-      <c r="D30" t="s">
-        <v>34</v>
-      </c>
-      <c r="E30" t="s">
-        <v>34</v>
-      </c>
-      <c r="F30" t="s">
-        <v>92</v>
-      </c>
       <c r="G30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H30" t="s">
         <v>34</v>
@@ -1887,33 +1869,33 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
+        <v>92</v>
+      </c>
+      <c r="B31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" t="s">
         <v>93</v>
       </c>
-      <c r="B31" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" t="s">
-        <v>10</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>94</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>95</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>96</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>97</v>
-      </c>
-      <c r="H31" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
@@ -1922,16 +1904,16 @@
         <v>10</v>
       </c>
       <c r="D32" t="s">
+        <v>54</v>
+      </c>
+      <c r="E32" t="s">
         <v>55</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>56</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>57</v>
-      </c>
-      <c r="G32" t="s">
-        <v>58</v>
       </c>
       <c r="H32" t="s">
         <v>34</v>
@@ -1939,7 +1921,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B33" t="s">
         <v>9</v>
@@ -1965,7 +1947,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
@@ -1986,30 +1968,30 @@
         <v>19</v>
       </c>
       <c r="H34" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
+        <v>101</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" t="s">
         <v>102</v>
       </c>
-      <c r="B35" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="E35" t="s">
         <v>103</v>
       </c>
-      <c r="E35" t="s">
+      <c r="F35" t="s">
         <v>104</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>105</v>
-      </c>
-      <c r="G35" t="s">
-        <v>106</v>
       </c>
       <c r="H35" t="s">
         <v>34</v>
@@ -2017,51 +1999,51 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
+        <v>106</v>
+      </c>
+      <c r="B36" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" t="s">
+        <v>46</v>
+      </c>
+      <c r="D36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E36" t="s">
+        <v>48</v>
+      </c>
+      <c r="F36" t="s">
+        <v>49</v>
+      </c>
+      <c r="G36" t="s">
+        <v>50</v>
+      </c>
+      <c r="H36" t="s">
         <v>107</v>
-      </c>
-      <c r="B36" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" t="s">
-        <v>47</v>
-      </c>
-      <c r="D36" t="s">
-        <v>48</v>
-      </c>
-      <c r="E36" t="s">
-        <v>49</v>
-      </c>
-      <c r="F36" t="s">
-        <v>50</v>
-      </c>
-      <c r="G36" t="s">
-        <v>51</v>
-      </c>
-      <c r="H36" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
+        <v>108</v>
+      </c>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>46</v>
+      </c>
+      <c r="D37" t="s">
         <v>109</v>
       </c>
-      <c r="B37" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" t="s">
-        <v>47</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>110</v>
       </c>
-      <c r="E37" t="s">
+      <c r="F37" t="s">
         <v>111</v>
       </c>
-      <c r="F37" t="s">
-        <v>112</v>
-      </c>
       <c r="G37" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H37" t="s">
         <v>34</v>
@@ -2069,7 +2051,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -2081,13 +2063,13 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
+        <v>68</v>
+      </c>
+      <c r="F38" t="s">
         <v>69</v>
       </c>
-      <c r="F38" t="s">
-        <v>70</v>
-      </c>
       <c r="G38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H38" t="s">
         <v>34</v>
@@ -2095,25 +2077,25 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
+        <v>114</v>
+      </c>
+      <c r="B39" t="s">
         <v>115</v>
       </c>
-      <c r="B39" t="s">
-        <v>34</v>
-      </c>
       <c r="C39" t="s">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="D39" t="s">
-        <v>34</v>
+        <v>117</v>
       </c>
       <c r="E39" t="s">
-        <v>34</v>
+        <v>118</v>
       </c>
       <c r="F39" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G39" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H39" t="s">
         <v>34</v>
@@ -2121,7 +2103,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
@@ -2147,7 +2129,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
@@ -2159,21 +2141,21 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
+        <v>60</v>
+      </c>
+      <c r="F41" t="s">
         <v>61</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>62</v>
       </c>
-      <c r="G41" t="s">
-        <v>63</v>
-      </c>
       <c r="H41" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -2199,7 +2181,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -2214,10 +2196,10 @@
         <v>34</v>
       </c>
       <c r="F43" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G43" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H43" t="s">
         <v>34</v>
@@ -2225,25 +2207,25 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
       </c>
       <c r="C44" t="s">
+        <v>46</v>
+      </c>
+      <c r="D44" t="s">
         <v>47</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>48</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>49</v>
       </c>
-      <c r="F44" t="s">
-        <v>50</v>
-      </c>
       <c r="G44" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H44" t="s">
         <v>34</v>
@@ -2251,7 +2233,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -2263,13 +2245,13 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
+        <v>68</v>
+      </c>
+      <c r="F45" t="s">
         <v>69</v>
       </c>
-      <c r="F45" t="s">
-        <v>70</v>
-      </c>
       <c r="G45" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H45" t="s">
         <v>34</v>
@@ -2277,7 +2259,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -2289,13 +2271,13 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
+        <v>60</v>
+      </c>
+      <c r="F46" t="s">
         <v>61</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>62</v>
-      </c>
-      <c r="G46" t="s">
-        <v>63</v>
       </c>
       <c r="H46" t="s">
         <v>34</v>
@@ -2303,33 +2285,33 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
       </c>
       <c r="C47" t="s">
+        <v>46</v>
+      </c>
+      <c r="D47" t="s">
         <v>47</v>
       </c>
-      <c r="D47" t="s">
-        <v>48</v>
-      </c>
       <c r="E47" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F47" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G47" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H47" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -2355,7 +2337,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -2381,7 +2363,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -2402,12 +2384,12 @@
         <v>19</v>
       </c>
       <c r="H50" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -2433,7 +2415,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B52" t="s">
         <v>9</v>
@@ -2445,21 +2427,21 @@
         <v>22</v>
       </c>
       <c r="E52" t="s">
+        <v>60</v>
+      </c>
+      <c r="F52" t="s">
         <v>61</v>
       </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
         <v>62</v>
       </c>
-      <c r="G52" t="s">
-        <v>63</v>
-      </c>
       <c r="H52" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -2480,12 +2462,12 @@
         <v>14</v>
       </c>
       <c r="H53" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B54" t="s">
         <v>9</v>
@@ -2494,50 +2476,50 @@
         <v>10</v>
       </c>
       <c r="D54" t="s">
+        <v>93</v>
+      </c>
+      <c r="E54" t="s">
         <v>94</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
         <v>95</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>96</v>
       </c>
-      <c r="G54" t="s">
-        <v>97</v>
-      </c>
       <c r="H54" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
       </c>
       <c r="C55" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D55" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E55" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F55" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="G55" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="H55" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B56" t="s">
         <v>9</v>
@@ -2558,30 +2540,30 @@
         <v>19</v>
       </c>
       <c r="H56" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B57" t="s">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="C57" t="s">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="D57" t="s">
-        <v>34</v>
+        <v>117</v>
       </c>
       <c r="E57" t="s">
-        <v>34</v>
+        <v>118</v>
       </c>
       <c r="F57" t="s">
-        <v>151</v>
+        <v>119</v>
       </c>
       <c r="G57" t="s">
-        <v>151</v>
+        <v>120</v>
       </c>
       <c r="H57" t="s">
         <v>34</v>
@@ -2589,7 +2571,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B58" t="s">
         <v>9</v>
@@ -2610,12 +2592,12 @@
         <v>19</v>
       </c>
       <c r="H58" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B59" t="s">
         <v>9</v>
@@ -2636,12 +2618,12 @@
         <v>19</v>
       </c>
       <c r="H59" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B60" t="s">
         <v>9</v>
@@ -2656,10 +2638,10 @@
         <v>29</v>
       </c>
       <c r="F60" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="G60" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="H60" t="s">
         <v>34</v>
@@ -2667,25 +2649,25 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="B61" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C61" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D61" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E61" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F61" t="s">
-        <v>157</v>
+        <v>18</v>
       </c>
       <c r="G61" t="s">
-        <v>157</v>
+        <v>19</v>
       </c>
       <c r="H61" t="s">
         <v>34</v>
@@ -2693,7 +2675,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B62" t="s">
         <v>9</v>
@@ -2705,21 +2687,21 @@
         <v>22</v>
       </c>
       <c r="E62" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F62" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G62" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H62" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B63" t="s">
         <v>9</v>
@@ -2740,30 +2722,30 @@
         <v>19</v>
       </c>
       <c r="H63" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B64" t="s">
         <v>9</v>
       </c>
       <c r="C64" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D64" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E64" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F64" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G64" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H64" t="s">
         <v>34</v>
@@ -2771,7 +2753,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B65" t="s">
         <v>9</v>
@@ -2792,38 +2774,38 @@
         <v>19</v>
       </c>
       <c r="H65" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B66" t="s">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="C66" t="s">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="D66" t="s">
-        <v>34</v>
+        <v>117</v>
       </c>
       <c r="E66" t="s">
-        <v>34</v>
+        <v>118</v>
       </c>
       <c r="F66" t="s">
-        <v>171</v>
+        <v>119</v>
       </c>
       <c r="G66" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H66" t="s">
-        <v>34</v>
+        <v>174</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B67" t="s">
         <v>9</v>
@@ -2849,7 +2831,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B68" t="s">
         <v>9</v>
@@ -2870,12 +2852,12 @@
         <v>19</v>
       </c>
       <c r="H68" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B69" t="s">
         <v>9</v>
@@ -2901,7 +2883,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B70" t="s">
         <v>9</v>
@@ -2916,10 +2898,10 @@
         <v>34</v>
       </c>
       <c r="F70" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="G70" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H70" t="s">
         <v>34</v>
@@ -2927,7 +2909,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B71" t="s">
         <v>9</v>
@@ -2936,16 +2918,16 @@
         <v>10</v>
       </c>
       <c r="D71" t="s">
+        <v>102</v>
+      </c>
+      <c r="E71" t="s">
         <v>103</v>
       </c>
-      <c r="E71" t="s">
-        <v>104</v>
-      </c>
       <c r="F71" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G71" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="H71" t="s">
         <v>34</v>
@@ -2953,7 +2935,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B72" t="s">
         <v>9</v>
@@ -2962,16 +2944,16 @@
         <v>10</v>
       </c>
       <c r="D72" t="s">
+        <v>102</v>
+      </c>
+      <c r="E72" t="s">
         <v>103</v>
       </c>
-      <c r="E72" t="s">
-        <v>104</v>
-      </c>
       <c r="F72" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="G72" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H72" t="s">
         <v>34</v>
@@ -2979,59 +2961,59 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B73" t="s">
         <v>9</v>
       </c>
       <c r="C73" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D73" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E73" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F73" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="G73" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="H73" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B74" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C74" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D74" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E74" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F74" t="s">
-        <v>191</v>
+        <v>18</v>
       </c>
       <c r="G74" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
       <c r="H74" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B75" t="s">
         <v>9</v>
@@ -3057,7 +3039,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B76" t="s">
         <v>9</v>
@@ -3078,38 +3060,38 @@
         <v>19</v>
       </c>
       <c r="H76" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B77" t="s">
         <v>9</v>
       </c>
       <c r="C77" t="s">
+        <v>46</v>
+      </c>
+      <c r="D77" t="s">
         <v>47</v>
       </c>
-      <c r="D77" t="s">
-        <v>48</v>
-      </c>
       <c r="E77" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="F77" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G77" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H77" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B78" t="s">
         <v>9</v>
@@ -3121,13 +3103,13 @@
         <v>22</v>
       </c>
       <c r="E78" t="s">
+        <v>60</v>
+      </c>
+      <c r="F78" t="s">
         <v>61</v>
       </c>
-      <c r="F78" t="s">
+      <c r="G78" t="s">
         <v>62</v>
-      </c>
-      <c r="G78" t="s">
-        <v>63</v>
       </c>
       <c r="H78" t="s">
         <v>34</v>
@@ -3135,7 +3117,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B79" t="s">
         <v>9</v>
@@ -3150,10 +3132,10 @@
         <v>34</v>
       </c>
       <c r="F79" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G79" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H79" t="s">
         <v>34</v>
@@ -3161,7 +3143,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B80" t="s">
         <v>9</v>
@@ -3182,12 +3164,12 @@
         <v>19</v>
       </c>
       <c r="H80" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B81" t="s">
         <v>9</v>
@@ -3199,21 +3181,21 @@
         <v>22</v>
       </c>
       <c r="E81" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F81" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G81" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H81" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B82" t="s">
         <v>9</v>
@@ -3239,7 +3221,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B83" t="s">
         <v>9</v>
@@ -3254,10 +3236,10 @@
         <v>34</v>
       </c>
       <c r="F83" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G83" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H83" t="s">
         <v>34</v>
@@ -3265,7 +3247,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B84" t="s">
         <v>9</v>
@@ -3286,12 +3268,12 @@
         <v>19</v>
       </c>
       <c r="H84" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B85" t="s">
         <v>9</v>
@@ -3312,12 +3294,12 @@
         <v>19</v>
       </c>
       <c r="H85" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B86" t="s">
         <v>9</v>
@@ -3343,51 +3325,51 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B87" t="s">
-        <v>34</v>
+        <v>115</v>
       </c>
       <c r="C87" t="s">
-        <v>34</v>
+        <v>116</v>
       </c>
       <c r="D87" t="s">
-        <v>34</v>
+        <v>117</v>
       </c>
       <c r="E87" t="s">
-        <v>34</v>
+        <v>118</v>
       </c>
       <c r="F87" t="s">
-        <v>212</v>
+        <v>119</v>
       </c>
       <c r="G87" t="s">
-        <v>212</v>
+        <v>120</v>
       </c>
       <c r="H87" t="s">
-        <v>34</v>
+        <v>214</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B88" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C88" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D88" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E88" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F88" t="s">
-        <v>214</v>
+        <v>18</v>
       </c>
       <c r="G88" t="s">
-        <v>214</v>
+        <v>19</v>
       </c>
       <c r="H88" t="s">
         <v>34</v>
@@ -3395,7 +3377,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B89" t="s">
         <v>9</v>
@@ -3416,12 +3398,12 @@
         <v>19</v>
       </c>
       <c r="H89" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B90" t="s">
         <v>9</v>
@@ -3430,16 +3412,16 @@
         <v>10</v>
       </c>
       <c r="D90" t="s">
+        <v>102</v>
+      </c>
+      <c r="E90" t="s">
         <v>103</v>
       </c>
-      <c r="E90" t="s">
-        <v>104</v>
-      </c>
       <c r="F90" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="G90" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H90" t="s">
         <v>34</v>
@@ -3447,7 +3429,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B91" t="s">
         <v>34</v>
@@ -3462,10 +3444,10 @@
         <v>34</v>
       </c>
       <c r="F91" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G91" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H91" t="s">
         <v>34</v>
@@ -3473,25 +3455,25 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B92" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C92" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D92" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E92" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F92" t="s">
-        <v>221</v>
+        <v>18</v>
       </c>
       <c r="G92" t="s">
-        <v>221</v>
+        <v>19</v>
       </c>
       <c r="H92" t="s">
         <v>34</v>
@@ -3520,7 +3502,7 @@
         <v>19</v>
       </c>
       <c r="H93" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="94">
@@ -3580,22 +3562,22 @@
         <v>227</v>
       </c>
       <c r="B96" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C96" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D96" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E96" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F96" t="s">
-        <v>228</v>
+        <v>18</v>
       </c>
       <c r="G96" t="s">
-        <v>228</v>
+        <v>19</v>
       </c>
       <c r="H96" t="s">
         <v>34</v>
@@ -3603,7 +3585,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B97" t="s">
         <v>9</v>
@@ -3618,10 +3600,10 @@
         <v>29</v>
       </c>
       <c r="F97" t="s">
+        <v>88</v>
+      </c>
+      <c r="G97" t="s">
         <v>89</v>
-      </c>
-      <c r="G97" t="s">
-        <v>90</v>
       </c>
       <c r="H97" t="s">
         <v>34</v>
@@ -3629,25 +3611,25 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B98" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C98" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D98" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E98" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F98" t="s">
-        <v>231</v>
+        <v>18</v>
       </c>
       <c r="G98" t="s">
-        <v>231</v>
+        <v>19</v>
       </c>
       <c r="H98" t="s">
         <v>34</v>
@@ -3655,7 +3637,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B99" t="s">
         <v>9</v>
@@ -3676,12 +3658,12 @@
         <v>19</v>
       </c>
       <c r="H99" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B100" t="s">
         <v>9</v>
@@ -3702,12 +3684,12 @@
         <v>19</v>
       </c>
       <c r="H100" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B101" t="s">
         <v>9</v>
@@ -3722,18 +3704,18 @@
         <v>23</v>
       </c>
       <c r="F101" t="s">
+        <v>233</v>
+      </c>
+      <c r="G101" t="s">
+        <v>234</v>
+      </c>
+      <c r="H101" t="s">
         <v>235</v>
-      </c>
-      <c r="G101" t="s">
-        <v>236</v>
-      </c>
-      <c r="H101" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B102" t="s">
         <v>9</v>
@@ -3754,30 +3736,30 @@
         <v>19</v>
       </c>
       <c r="H102" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B103" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C103" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D103" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E103" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F103" t="s">
-        <v>240</v>
+        <v>18</v>
       </c>
       <c r="G103" t="s">
-        <v>240</v>
+        <v>19</v>
       </c>
       <c r="H103" t="s">
         <v>34</v>
@@ -3785,25 +3767,25 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B104" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C104" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D104" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E104" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F104" t="s">
-        <v>242</v>
+        <v>18</v>
       </c>
       <c r="G104" t="s">
-        <v>242</v>
+        <v>19</v>
       </c>
       <c r="H104" t="s">
         <v>34</v>
@@ -3811,7 +3793,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B105" t="s">
         <v>9</v>
@@ -3826,10 +3808,10 @@
         <v>29</v>
       </c>
       <c r="F105" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="G105" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="H105" t="s">
         <v>34</v>
@@ -3837,25 +3819,25 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B106" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C106" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D106" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E106" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F106" t="s">
-        <v>246</v>
+        <v>18</v>
       </c>
       <c r="G106" t="s">
-        <v>246</v>
+        <v>19</v>
       </c>
       <c r="H106" t="s">
         <v>34</v>
@@ -3863,7 +3845,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B107" t="s">
         <v>9</v>
@@ -3884,12 +3866,12 @@
         <v>19</v>
       </c>
       <c r="H107" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B108" t="s">
         <v>9</v>
@@ -3904,10 +3886,10 @@
         <v>34</v>
       </c>
       <c r="F108" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="G108" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="H108" t="s">
         <v>34</v>
@@ -3915,7 +3897,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="B109" t="s">
         <v>9</v>
@@ -3936,38 +3918,38 @@
         <v>19</v>
       </c>
       <c r="H109" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B110" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C110" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D110" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E110" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F110" t="s">
-        <v>252</v>
+        <v>18</v>
       </c>
       <c r="G110" t="s">
-        <v>252</v>
+        <v>19</v>
       </c>
       <c r="H110" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B111" t="s">
         <v>9</v>
@@ -3988,12 +3970,12 @@
         <v>19</v>
       </c>
       <c r="H111" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="B112" t="s">
         <v>9</v>
@@ -4005,16 +3987,16 @@
         <v>22</v>
       </c>
       <c r="E112" t="s">
+        <v>60</v>
+      </c>
+      <c r="F112" t="s">
         <v>61</v>
       </c>
-      <c r="F112" t="s">
+      <c r="G112" t="s">
         <v>62</v>
       </c>
-      <c r="G112" t="s">
-        <v>63</v>
-      </c>
       <c r="H112" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>